<commit_message>
active inactive option enab led
</commit_message>
<xml_diff>
--- a/Documents/Product Catalog/Bedroom Set Uv Print.xlsx
+++ b/Documents/Product Catalog/Bedroom Set Uv Print.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Talukder Furniture\Documents\Product Catalog\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2417B5D2-347E-447B-A6F4-AE9DB17323F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C1BAD79-90EF-41E0-A657-AAF5F12F1A41}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="437" uniqueCount="133">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="437" uniqueCount="135">
   <si>
     <t>Home Furniture Specifications</t>
   </si>
@@ -548,12 +548,18 @@
   <si>
     <t xml:space="preserve">Bed side Table </t>
   </si>
+  <si>
+    <t>TFL-COD-119 LB</t>
+  </si>
+  <si>
+    <t>TFL-COD-120 LB</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
-  <fonts count="9">
+  <fonts count="12">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -608,6 +614,21 @@
       <color theme="1"/>
       <name val="Times New Roman"/>
       <charset val="134"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="16"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
     </font>
   </fonts>
   <fills count="5">
@@ -805,7 +826,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="52">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -888,9 +909,6 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -912,11 +930,56 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="9" fillId="0" borderId="9" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="10" fillId="3" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="10" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="10" fillId="4" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2226,7 +2289,7 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="4511606" y="24153825"/>
+          <a:off x="4510369" y="24219387"/>
           <a:ext cx="682117" cy="930695"/>
           <a:chOff x="0" y="0"/>
           <a:chExt cx="409575" cy="567055"/>
@@ -2445,7 +2508,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="4419854" y="182818964"/>
+          <a:off x="4430740" y="27262107"/>
           <a:ext cx="653796" cy="937336"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -3126,55 +3189,55 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:46" ht="39.950000000000003" customHeight="1">
-      <c r="A1" s="32" t="s">
+      <c r="A1" s="31" t="s">
         <v>122</v>
       </c>
-      <c r="B1" s="32"/>
-      <c r="C1" s="32"/>
-      <c r="D1" s="32"/>
-      <c r="E1" s="32"/>
-      <c r="F1" s="32"/>
-      <c r="G1" s="32"/>
-      <c r="H1" s="32"/>
-      <c r="I1" s="32"/>
-      <c r="J1" s="32"/>
-      <c r="K1" s="32"/>
-      <c r="L1" s="32"/>
-      <c r="M1" s="32"/>
-      <c r="N1" s="32"/>
-      <c r="O1" s="32"/>
-      <c r="P1" s="32"/>
-      <c r="Q1" s="32"/>
+      <c r="B1" s="31"/>
+      <c r="C1" s="31"/>
+      <c r="D1" s="31"/>
+      <c r="E1" s="31"/>
+      <c r="F1" s="31"/>
+      <c r="G1" s="31"/>
+      <c r="H1" s="31"/>
+      <c r="I1" s="31"/>
+      <c r="J1" s="31"/>
+      <c r="K1" s="31"/>
+      <c r="L1" s="31"/>
+      <c r="M1" s="31"/>
+      <c r="N1" s="31"/>
+      <c r="O1" s="31"/>
+      <c r="P1" s="31"/>
+      <c r="Q1" s="31"/>
     </row>
     <row r="2" spans="1:46" ht="39.950000000000003" customHeight="1">
-      <c r="A2" s="33" t="s">
+      <c r="A2" s="32" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="33"/>
-      <c r="C2" s="33"/>
-      <c r="D2" s="33"/>
-      <c r="E2" s="33"/>
-      <c r="F2" s="33"/>
-      <c r="G2" s="33"/>
-      <c r="H2" s="33"/>
-      <c r="I2" s="33"/>
-      <c r="J2" s="33"/>
-      <c r="K2" s="33"/>
-      <c r="L2" s="33"/>
-      <c r="M2" s="33"/>
-      <c r="N2" s="33"/>
-      <c r="O2" s="33"/>
-      <c r="P2" s="33"/>
-      <c r="Q2" s="33"/>
+      <c r="B2" s="32"/>
+      <c r="C2" s="32"/>
+      <c r="D2" s="32"/>
+      <c r="E2" s="32"/>
+      <c r="F2" s="32"/>
+      <c r="G2" s="32"/>
+      <c r="H2" s="32"/>
+      <c r="I2" s="32"/>
+      <c r="J2" s="32"/>
+      <c r="K2" s="32"/>
+      <c r="L2" s="32"/>
+      <c r="M2" s="32"/>
+      <c r="N2" s="32"/>
+      <c r="O2" s="32"/>
+      <c r="P2" s="32"/>
+      <c r="Q2" s="32"/>
     </row>
     <row r="3" spans="1:46" ht="50.1" customHeight="1">
-      <c r="A3" s="34" t="s">
+      <c r="A3" s="33" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="28" t="s">
+      <c r="B3" s="35" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="28" t="s">
+      <c r="C3" s="35" t="s">
         <v>3</v>
       </c>
       <c r="D3" s="36" t="s">
@@ -3183,32 +3246,32 @@
       <c r="E3" s="36" t="s">
         <v>5</v>
       </c>
-      <c r="F3" s="29" t="s">
+      <c r="F3" s="28" t="s">
         <v>6</v>
       </c>
-      <c r="G3" s="30"/>
-      <c r="H3" s="31"/>
-      <c r="I3" s="28" t="s">
+      <c r="G3" s="29"/>
+      <c r="H3" s="30"/>
+      <c r="I3" s="35" t="s">
         <v>7</v>
       </c>
       <c r="J3" s="36" t="s">
         <v>8</v>
       </c>
-      <c r="K3" s="28" t="s">
+      <c r="K3" s="35" t="s">
         <v>9</v>
       </c>
-      <c r="L3" s="28"/>
-      <c r="M3" s="29"/>
-      <c r="N3" s="28" t="s">
+      <c r="L3" s="35"/>
+      <c r="M3" s="28"/>
+      <c r="N3" s="35" t="s">
         <v>10</v>
       </c>
-      <c r="O3" s="28" t="s">
+      <c r="O3" s="35" t="s">
         <v>11</v>
       </c>
-      <c r="P3" s="28" t="s">
+      <c r="P3" s="35" t="s">
         <v>103</v>
       </c>
-      <c r="Q3" s="28" t="s">
+      <c r="Q3" s="35" t="s">
         <v>88</v>
       </c>
       <c r="S3" s="4"/>
@@ -3241,9 +3304,9 @@
       <c r="AT3" s="4"/>
     </row>
     <row r="4" spans="1:46" ht="33.200000000000003" customHeight="1">
-      <c r="A4" s="35"/>
-      <c r="B4" s="28"/>
-      <c r="C4" s="28"/>
+      <c r="A4" s="34"/>
+      <c r="B4" s="35"/>
+      <c r="C4" s="35"/>
       <c r="D4" s="37"/>
       <c r="E4" s="37"/>
       <c r="F4" s="27" t="s">
@@ -3255,7 +3318,7 @@
       <c r="H4" s="27" t="s">
         <v>131</v>
       </c>
-      <c r="I4" s="28"/>
+      <c r="I4" s="35"/>
       <c r="J4" s="37"/>
       <c r="K4" s="5" t="s">
         <v>14</v>
@@ -3266,10 +3329,10 @@
       <c r="M4" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="N4" s="28"/>
-      <c r="O4" s="28"/>
-      <c r="P4" s="28"/>
-      <c r="Q4" s="28"/>
+      <c r="N4" s="35"/>
+      <c r="O4" s="35"/>
+      <c r="P4" s="35"/>
+      <c r="Q4" s="35"/>
       <c r="S4" s="4"/>
       <c r="T4" s="4"/>
       <c r="U4" s="4"/>
@@ -5299,245 +5362,245 @@
       <c r="AS29" s="1"/>
       <c r="AT29" s="1"/>
     </row>
-    <row r="30" spans="1:46" s="4" customFormat="1" ht="80.099999999999994" customHeight="1">
-      <c r="A30" s="21" t="s">
+    <row r="30" spans="1:46" s="50" customFormat="1" ht="80.099999999999994" customHeight="1">
+      <c r="A30" s="38" t="s">
         <v>49</v>
       </c>
-      <c r="B30" s="7" t="s">
+      <c r="B30" s="39" t="s">
         <v>96</v>
       </c>
-      <c r="C30" s="7" t="s">
+      <c r="C30" s="39" t="s">
+        <v>83</v>
+      </c>
+      <c r="D30" s="39"/>
+      <c r="E30" s="40" t="s">
+        <v>57</v>
+      </c>
+      <c r="F30" s="41" t="s">
+        <v>19</v>
+      </c>
+      <c r="G30" s="42" t="s">
+        <v>20</v>
+      </c>
+      <c r="H30" s="42" t="s">
         <v>86</v>
       </c>
-      <c r="D30" s="8"/>
-      <c r="E30" s="9" t="s">
-        <v>57</v>
-      </c>
-      <c r="F30" s="10" t="s">
-        <v>19</v>
-      </c>
-      <c r="G30" s="11" t="s">
-        <v>20</v>
-      </c>
-      <c r="H30" s="11" t="s">
-        <v>86</v>
-      </c>
-      <c r="I30" s="12" t="s">
+      <c r="I30" s="43" t="s">
         <v>87</v>
       </c>
-      <c r="J30" s="12" t="s">
+      <c r="J30" s="43" t="s">
         <v>80</v>
       </c>
-      <c r="K30" s="13">
+      <c r="K30" s="44">
         <f t="shared" si="0"/>
         <v>15750</v>
       </c>
-      <c r="L30" s="17">
+      <c r="L30" s="45">
         <v>17500</v>
       </c>
-      <c r="M30" s="15">
+      <c r="M30" s="46">
         <v>0.1</v>
       </c>
-      <c r="N30" s="22" t="s">
+      <c r="N30" s="47" t="s">
         <v>114</v>
       </c>
-      <c r="O30" s="24" t="s">
+      <c r="O30" s="48" t="s">
         <v>115</v>
       </c>
-      <c r="P30" s="23" t="s">
+      <c r="P30" s="49" t="s">
         <v>116</v>
       </c>
-      <c r="Q30" s="23" t="s">
+      <c r="Q30" s="49" t="s">
         <v>102</v>
       </c>
-      <c r="S30" s="1"/>
-      <c r="T30" s="1"/>
-      <c r="U30" s="1"/>
-      <c r="V30" s="1"/>
-      <c r="W30" s="1"/>
-      <c r="X30" s="1"/>
-      <c r="Y30" s="1"/>
-      <c r="Z30" s="1"/>
-      <c r="AA30" s="1"/>
-      <c r="AB30" s="1"/>
-      <c r="AC30" s="1"/>
-      <c r="AD30" s="1"/>
-      <c r="AE30" s="1"/>
-      <c r="AF30" s="1"/>
-      <c r="AG30" s="1"/>
-      <c r="AH30" s="1"/>
-      <c r="AI30" s="1"/>
-      <c r="AJ30" s="1"/>
-      <c r="AK30" s="1"/>
-      <c r="AL30" s="1"/>
-      <c r="AM30" s="1"/>
-      <c r="AN30" s="1"/>
-      <c r="AO30" s="1"/>
-      <c r="AP30" s="1"/>
-      <c r="AQ30" s="1"/>
-      <c r="AR30" s="1"/>
-      <c r="AS30" s="1"/>
-      <c r="AT30" s="1"/>
-    </row>
-    <row r="31" spans="1:46" s="4" customFormat="1" ht="80.099999999999994" customHeight="1">
-      <c r="A31" s="21" t="s">
+      <c r="S30" s="51"/>
+      <c r="T30" s="51"/>
+      <c r="U30" s="51"/>
+      <c r="V30" s="51"/>
+      <c r="W30" s="51"/>
+      <c r="X30" s="51"/>
+      <c r="Y30" s="51"/>
+      <c r="Z30" s="51"/>
+      <c r="AA30" s="51"/>
+      <c r="AB30" s="51"/>
+      <c r="AC30" s="51"/>
+      <c r="AD30" s="51"/>
+      <c r="AE30" s="51"/>
+      <c r="AF30" s="51"/>
+      <c r="AG30" s="51"/>
+      <c r="AH30" s="51"/>
+      <c r="AI30" s="51"/>
+      <c r="AJ30" s="51"/>
+      <c r="AK30" s="51"/>
+      <c r="AL30" s="51"/>
+      <c r="AM30" s="51"/>
+      <c r="AN30" s="51"/>
+      <c r="AO30" s="51"/>
+      <c r="AP30" s="51"/>
+      <c r="AQ30" s="51"/>
+      <c r="AR30" s="51"/>
+      <c r="AS30" s="51"/>
+      <c r="AT30" s="51"/>
+    </row>
+    <row r="31" spans="1:46" s="50" customFormat="1" ht="80.099999999999994" customHeight="1">
+      <c r="A31" s="38" t="s">
         <v>50</v>
       </c>
-      <c r="B31" s="7" t="s">
-        <v>91</v>
-      </c>
-      <c r="C31" s="7" t="s">
+      <c r="B31" s="39" t="s">
+        <v>133</v>
+      </c>
+      <c r="C31" s="39" t="s">
         <v>86</v>
       </c>
-      <c r="D31" s="8"/>
-      <c r="E31" s="9" t="s">
+      <c r="D31" s="39"/>
+      <c r="E31" s="40" t="s">
         <v>57</v>
       </c>
-      <c r="F31" s="10" t="s">
+      <c r="F31" s="41" t="s">
         <v>19</v>
       </c>
-      <c r="G31" s="11" t="s">
+      <c r="G31" s="42" t="s">
         <v>20</v>
       </c>
-      <c r="H31" s="11" t="s">
+      <c r="H31" s="42" t="s">
         <v>86</v>
       </c>
-      <c r="I31" s="12" t="s">
+      <c r="I31" s="43" t="s">
         <v>84</v>
       </c>
-      <c r="J31" s="12" t="s">
+      <c r="J31" s="43" t="s">
         <v>80</v>
       </c>
-      <c r="K31" s="13">
+      <c r="K31" s="44">
         <f t="shared" si="0"/>
         <v>15750</v>
       </c>
-      <c r="L31" s="17">
+      <c r="L31" s="45">
         <v>17500</v>
       </c>
-      <c r="M31" s="15">
+      <c r="M31" s="46">
         <v>0.1</v>
       </c>
-      <c r="N31" s="22" t="s">
+      <c r="N31" s="47" t="s">
         <v>117</v>
       </c>
-      <c r="O31" s="24" t="s">
+      <c r="O31" s="48" t="s">
         <v>115</v>
       </c>
-      <c r="P31" s="23" t="s">
+      <c r="P31" s="49" t="s">
         <v>116</v>
       </c>
-      <c r="Q31" s="23" t="s">
+      <c r="Q31" s="49" t="s">
         <v>102</v>
       </c>
-      <c r="S31" s="1"/>
-      <c r="T31" s="1"/>
-      <c r="U31" s="1"/>
-      <c r="V31" s="1"/>
-      <c r="W31" s="1"/>
-      <c r="X31" s="1"/>
-      <c r="Y31" s="1"/>
-      <c r="Z31" s="1"/>
-      <c r="AA31" s="1"/>
-      <c r="AB31" s="1"/>
-      <c r="AC31" s="1"/>
-      <c r="AD31" s="1"/>
-      <c r="AE31" s="1"/>
-      <c r="AF31" s="1"/>
-      <c r="AG31" s="1"/>
-      <c r="AH31" s="1"/>
-      <c r="AI31" s="1"/>
-      <c r="AJ31" s="1"/>
-      <c r="AK31" s="1"/>
-      <c r="AL31" s="1"/>
-      <c r="AM31" s="1"/>
-      <c r="AN31" s="1"/>
-      <c r="AO31" s="1"/>
-      <c r="AP31" s="1"/>
-      <c r="AQ31" s="1"/>
-      <c r="AR31" s="1"/>
-      <c r="AS31" s="1"/>
-      <c r="AT31" s="1"/>
-    </row>
-    <row r="32" spans="1:46" s="4" customFormat="1" ht="80.099999999999994" customHeight="1">
-      <c r="A32" s="21" t="s">
+      <c r="S31" s="51"/>
+      <c r="T31" s="51"/>
+      <c r="U31" s="51"/>
+      <c r="V31" s="51"/>
+      <c r="W31" s="51"/>
+      <c r="X31" s="51"/>
+      <c r="Y31" s="51"/>
+      <c r="Z31" s="51"/>
+      <c r="AA31" s="51"/>
+      <c r="AB31" s="51"/>
+      <c r="AC31" s="51"/>
+      <c r="AD31" s="51"/>
+      <c r="AE31" s="51"/>
+      <c r="AF31" s="51"/>
+      <c r="AG31" s="51"/>
+      <c r="AH31" s="51"/>
+      <c r="AI31" s="51"/>
+      <c r="AJ31" s="51"/>
+      <c r="AK31" s="51"/>
+      <c r="AL31" s="51"/>
+      <c r="AM31" s="51"/>
+      <c r="AN31" s="51"/>
+      <c r="AO31" s="51"/>
+      <c r="AP31" s="51"/>
+      <c r="AQ31" s="51"/>
+      <c r="AR31" s="51"/>
+      <c r="AS31" s="51"/>
+      <c r="AT31" s="51"/>
+    </row>
+    <row r="32" spans="1:46" s="50" customFormat="1" ht="80.099999999999994" customHeight="1">
+      <c r="A32" s="38" t="s">
         <v>51</v>
       </c>
-      <c r="B32" s="7" t="s">
-        <v>92</v>
-      </c>
-      <c r="C32" s="7" t="s">
+      <c r="B32" s="39" t="s">
+        <v>134</v>
+      </c>
+      <c r="C32" s="39" t="s">
         <v>86</v>
       </c>
-      <c r="D32" s="8"/>
-      <c r="E32" s="9" t="s">
+      <c r="D32" s="39"/>
+      <c r="E32" s="40" t="s">
         <v>57</v>
       </c>
-      <c r="F32" s="10" t="s">
+      <c r="F32" s="41" t="s">
         <v>19</v>
       </c>
-      <c r="G32" s="11" t="s">
+      <c r="G32" s="42" t="s">
         <v>20</v>
       </c>
-      <c r="H32" s="11" t="s">
+      <c r="H32" s="42" t="s">
         <v>86</v>
       </c>
-      <c r="I32" s="12" t="s">
+      <c r="I32" s="43" t="s">
         <v>87</v>
       </c>
-      <c r="J32" s="12" t="s">
+      <c r="J32" s="43" t="s">
         <v>80</v>
       </c>
-      <c r="K32" s="13">
+      <c r="K32" s="44">
         <f t="shared" si="0"/>
         <v>15750</v>
       </c>
-      <c r="L32" s="17">
+      <c r="L32" s="45">
         <v>17500</v>
       </c>
-      <c r="M32" s="15">
+      <c r="M32" s="46">
         <v>0.1</v>
       </c>
-      <c r="N32" s="22" t="s">
+      <c r="N32" s="47" t="s">
         <v>118</v>
       </c>
-      <c r="O32" s="24" t="s">
+      <c r="O32" s="48" t="s">
         <v>115</v>
       </c>
-      <c r="P32" s="23" t="s">
+      <c r="P32" s="49" t="s">
         <v>116</v>
       </c>
-      <c r="Q32" s="23" t="s">
+      <c r="Q32" s="49" t="s">
         <v>102</v>
       </c>
-      <c r="S32" s="1"/>
-      <c r="T32" s="1"/>
-      <c r="U32" s="1"/>
-      <c r="V32" s="1"/>
-      <c r="W32" s="1"/>
-      <c r="X32" s="1"/>
-      <c r="Y32" s="1"/>
-      <c r="Z32" s="1"/>
-      <c r="AA32" s="1"/>
-      <c r="AB32" s="1"/>
-      <c r="AC32" s="1"/>
-      <c r="AD32" s="1"/>
-      <c r="AE32" s="1"/>
-      <c r="AF32" s="1"/>
-      <c r="AG32" s="1"/>
-      <c r="AH32" s="1"/>
-      <c r="AI32" s="1"/>
-      <c r="AJ32" s="1"/>
-      <c r="AK32" s="1"/>
-      <c r="AL32" s="1"/>
-      <c r="AM32" s="1"/>
-      <c r="AN32" s="1"/>
-      <c r="AO32" s="1"/>
-      <c r="AP32" s="1"/>
-      <c r="AQ32" s="1"/>
-      <c r="AR32" s="1"/>
-      <c r="AS32" s="1"/>
-      <c r="AT32" s="1"/>
+      <c r="S32" s="51"/>
+      <c r="T32" s="51"/>
+      <c r="U32" s="51"/>
+      <c r="V32" s="51"/>
+      <c r="W32" s="51"/>
+      <c r="X32" s="51"/>
+      <c r="Y32" s="51"/>
+      <c r="Z32" s="51"/>
+      <c r="AA32" s="51"/>
+      <c r="AB32" s="51"/>
+      <c r="AC32" s="51"/>
+      <c r="AD32" s="51"/>
+      <c r="AE32" s="51"/>
+      <c r="AF32" s="51"/>
+      <c r="AG32" s="51"/>
+      <c r="AH32" s="51"/>
+      <c r="AI32" s="51"/>
+      <c r="AJ32" s="51"/>
+      <c r="AK32" s="51"/>
+      <c r="AL32" s="51"/>
+      <c r="AM32" s="51"/>
+      <c r="AN32" s="51"/>
+      <c r="AO32" s="51"/>
+      <c r="AP32" s="51"/>
+      <c r="AQ32" s="51"/>
+      <c r="AR32" s="51"/>
+      <c r="AS32" s="51"/>
+      <c r="AT32" s="51"/>
     </row>
     <row r="33" spans="1:46" s="4" customFormat="1" ht="87" customHeight="1">
       <c r="A33" s="21" t="s">

</xml_diff>